<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:42:16)
</commit_message>
<xml_diff>
--- a/Talabalar_Yangilangan_Royxat.xlsx
+++ b/Talabalar_Yangilangan_Royxat.xlsx
@@ -10580,7 +10580,7 @@
       </c>
       <c r="R91" s="11" t="inlineStr">
         <is>
-          <t>OLCHOV-1</t>
+          <t>BATCH-C</t>
         </is>
       </c>
       <c r="S91" s="12" t="inlineStr">
@@ -29555,7 +29555,7 @@
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>OLCHOV-1</t>
+          <t>BATCH-C</t>
         </is>
       </c>
       <c r="S18" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 16:32:52)
</commit_message>
<xml_diff>
--- a/Talabalar_Yangilangan_Royxat.xlsx
+++ b/Talabalar_Yangilangan_Royxat.xlsx
@@ -8432,9 +8432,9 @@
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X71" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X71" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29847,9 +29847,9 @@
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X15" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X15" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 16:33:57)
</commit_message>
<xml_diff>
--- a/Talabalar_Yangilangan_Royxat.xlsx
+++ b/Talabalar_Yangilangan_Royxat.xlsx
@@ -17779,9 +17779,9 @@
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X158" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X158" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31118,9 +31118,9 @@
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X27" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X27" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 16:38:25)
</commit_message>
<xml_diff>
--- a/Talabalar_Yangilangan_Royxat.xlsx
+++ b/Talabalar_Yangilangan_Royxat.xlsx
@@ -12130,9 +12130,9 @@
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X106" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X106" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30285,9 +30285,9 @@
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X19" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X19" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 14:52:36)
</commit_message>
<xml_diff>
--- a/Talabalar_Yangilangan_Royxat.xlsx
+++ b/Talabalar_Yangilangan_Royxat.xlsx
@@ -14005,7 +14005,7 @@
       </c>
       <c r="K124" s="2" t="inlineStr">
         <is>
-          <t>28071542703279</t>
+          <t>41507985590024</t>
         </is>
       </c>
       <c r="L124" s="5" t="inlineStr">
@@ -14018,7 +14018,11 @@
           <t>15.07.1998</t>
         </is>
       </c>
-      <c r="N124" s="5" t="inlineStr"/>
+      <c r="N124" s="5" t="inlineStr">
+        <is>
+          <t>Shahrisabz tumani</t>
+        </is>
+      </c>
       <c r="O124" s="4" t="inlineStr">
         <is>
           <t>Mavjud</t>
@@ -38875,7 +38879,7 @@
       </c>
       <c r="K29" s="9" t="inlineStr">
         <is>
-          <t>28071542703279</t>
+          <t>41507985590024</t>
         </is>
       </c>
       <c r="L29" s="12" t="inlineStr">
@@ -38888,7 +38892,11 @@
           <t>15.07.1998</t>
         </is>
       </c>
-      <c r="N29" s="12" t="inlineStr"/>
+      <c r="N29" s="12" t="inlineStr">
+        <is>
+          <t>Shahrisabz tumani</t>
+        </is>
+      </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
           <t>Mavjud</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:36:35)
</commit_message>
<xml_diff>
--- a/Talabalar_Yangilangan_Royxat.xlsx
+++ b/Talabalar_Yangilangan_Royxat.xlsx
@@ -17386,9 +17386,9 @@
           <t>Pasport: MOS</t>
         </is>
       </c>
-      <c r="X150" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X150" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28868,9 +28868,9 @@
           <t>Pasport: MOS</t>
         </is>
       </c>
-      <c r="X26" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X26" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 10:33:02)
</commit_message>
<xml_diff>
--- a/Talabalar_Yangilangan_Royxat.xlsx
+++ b/Talabalar_Yangilangan_Royxat.xlsx
@@ -7051,7 +7051,7 @@
       </c>
       <c r="S57" s="12" t="inlineStr">
         <is>
-          <t>Kollej</t>
+          <t>Diplom</t>
         </is>
       </c>
       <c r="T57" s="12" t="inlineStr">
@@ -34938,7 +34938,7 @@
       </c>
       <c r="S13" s="12" t="inlineStr">
         <is>
-          <t>Kollej</t>
+          <t>Diplom</t>
         </is>
       </c>
       <c r="T13" s="12" t="inlineStr">

</xml_diff>